<commit_message>
CORRECTION: East West Bank is a MIXED program, not flatly Elan
One Card (business/corporate) = Elan per East West's own verbatim disclosure, BUT the bank
self-issues its Secured Visa Classic and holds $4.631M credit-card loans on its own books
(FDIC call report 2026-03-31, CERT 31628). Blanket 'Elan' label was wrong; flagged MIXED.

https://claude.ai/code/session_014WdfNSevF6i6PT6GydKC2F
</commit_message>
<xml_diff>
--- a/research/alameda/deliverables/Alameda_Oakland_NoDoc_NoSeasoning_v1.xlsx
+++ b/research/alameda/deliverables/Alameda_Oakland_NoDoc_NoSeasoning_v1.xlsx
@@ -507,9 +507,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -545,9 +543,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -590,9 +586,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -1268,7 +1262,7 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>https://www.eastwestbank.com/en/small-mid-size-businesses/corporate-card</t>
+          <t>https://www.eastwestbank.com/en/small-mid-size-businesses/corporate-card | MIXED PROGRAM (corrected 2026-07-26): the One Card (corporate/business) is Elan per East West's own page — "The creditor and issuer of the East West Bank One Card is Elan Financial Services, pursuant to a license from Visa U.S.A." BUT East West SELF-ISSUES its Secured Visa Classic (consumer; Elan not named) and books $4,631K of credit-card loans on its own balance sheet (FDIC call report 2026-03-31, CERT 31628). Do NOT label the bank flatly "Elan".</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4592,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fremont; Newark; Oakland; Pleasanton</t>
+          <t>Fremont; Newark; Oakland; Pleasanton | MIXED PROGRAM (corrected 2026-07-26): the One Card (corporate/business) is Elan per East West's own page — "The creditor and issuer of the East West Bank One Card is Elan Financial Services, pursuant to a license from Visa U.S.A." BUT East West SELF-ISSUES its Secured Visa Classic (consumer; Elan not named) and books $4,631K of credit-card loans on its own balance sheet (FDIC call report 2026-03-31, CERT 31628). Do NOT label the bank flatly "Elan".</t>
         </is>
       </c>
     </row>

</xml_diff>